<commit_message>
KCP-77 - wip (models master)
</commit_message>
<xml_diff>
--- a/resources/kcp-models-master.xlsx
+++ b/resources/kcp-models-master.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28122"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2F0C72ED-C198-4D55-8763-79CAA4ABE3C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{70E85B90-2538-4DE0-8EDA-C110139F2379}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080" firstSheet="6" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="125">
   <si>
     <t>Notes</t>
   </si>
@@ -468,10 +468,37 @@
     <t>Yes</t>
   </si>
   <si>
+    <t>:age-at-surgery</t>
+  </si>
+  <si>
+    <t>Age at surgery</t>
+  </si>
+  <si>
+    <t>:numeric</t>
+  </si>
+  <si>
+    <t>Age when the kidney cancer surgery was performed. An age between 25 and 85 may be entered here.</t>
+  </si>
+  <si>
+    <t>:sex</t>
+  </si>
+  <si>
+    <t>:male</t>
+  </si>
+  <si>
+    <t>Sex</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>:female</t>
+  </si>
+  <si>
+    <t>Female</t>
+  </si>
+  <si>
     <t>Age</t>
-  </si>
-  <si>
-    <t>Sex</t>
   </si>
   <si>
     <t>Year1</t>
@@ -4127,10 +4154,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:N24"/>
+  <dimension ref="A1:N27"/>
   <sheetFormatPr defaultColWidth="8.44140625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="8" style="1" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="10.33203125" style="1" customWidth="1"/>
     <col min="3" max="3" width="31" style="1" customWidth="1"/>
     <col min="4" max="4" width="43" style="1" customWidth="1"/>
@@ -4883,6 +4910,98 @@
         <v>1</v>
       </c>
     </row>
+    <row r="25" spans="1:14" ht="15.75" customHeight="1">
+      <c r="A25" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="B25" s="9"/>
+      <c r="C25" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="D25" s="9"/>
+      <c r="E25" s="25"/>
+      <c r="F25" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="G25" s="4"/>
+      <c r="H25" s="49" t="s">
+        <v>105</v>
+      </c>
+      <c r="I25" s="25">
+        <v>100</v>
+      </c>
+      <c r="J25" s="4"/>
+      <c r="K25" s="4"/>
+      <c r="L25" s="9"/>
+      <c r="M25" s="4"/>
+      <c r="N25" s="44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" ht="15.75" customHeight="1">
+      <c r="A26" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="E26" s="25"/>
+      <c r="F26" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="G26" s="4"/>
+      <c r="H26" s="49"/>
+      <c r="I26" s="25">
+        <v>110</v>
+      </c>
+      <c r="J26" s="4"/>
+      <c r="K26" s="4"/>
+      <c r="L26" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="M26" s="4"/>
+      <c r="N26" s="44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" ht="15.75" customHeight="1">
+      <c r="A27" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="C27" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="D27" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="E27" s="25"/>
+      <c r="F27" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="G27" s="4"/>
+      <c r="H27" s="49"/>
+      <c r="I27" s="25">
+        <v>110</v>
+      </c>
+      <c r="J27" s="4"/>
+      <c r="K27" s="4"/>
+      <c r="L27" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="M27" s="4"/>
+      <c r="N27" s="44">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51181100000000002" footer="0.51181100000000002"/>
   <pageSetup orientation="portrait"/>
@@ -4899,40 +5018,40 @@
   <sheetData>
     <row r="1" spans="1:12" ht="15.75">
       <c r="A1" s="50" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="B1" s="50" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="C1" s="50" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="D1" s="50" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="E1" s="50" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="F1" s="50" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="G1" s="50" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="H1" s="50" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="I1" s="50" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="J1" s="50" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="K1" s="50" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="L1" s="50" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2" spans="1:12">
@@ -4940,7 +5059,7 @@
         <v>25</v>
       </c>
       <c r="B2" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C2" s="51">
         <v>0</v>
@@ -4978,7 +5097,7 @@
         <v>26</v>
       </c>
       <c r="B3" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C3" s="51">
         <v>0</v>
@@ -5016,7 +5135,7 @@
         <v>27</v>
       </c>
       <c r="B4" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C4" s="51">
         <v>0</v>
@@ -5054,7 +5173,7 @@
         <v>28</v>
       </c>
       <c r="B5" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C5" s="51">
         <v>0</v>
@@ -5092,7 +5211,7 @@
         <v>29</v>
       </c>
       <c r="B6" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C6" s="51">
         <v>0</v>
@@ -5130,7 +5249,7 @@
         <v>30</v>
       </c>
       <c r="B7" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C7" s="51">
         <v>0</v>
@@ -5168,7 +5287,7 @@
         <v>31</v>
       </c>
       <c r="B8" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C8" s="51">
         <v>0</v>
@@ -5206,7 +5325,7 @@
         <v>32</v>
       </c>
       <c r="B9" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C9" s="51">
         <v>0</v>
@@ -5244,7 +5363,7 @@
         <v>33</v>
       </c>
       <c r="B10" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C10" s="51">
         <v>0</v>
@@ -5282,7 +5401,7 @@
         <v>34</v>
       </c>
       <c r="B11" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C11" s="51">
         <v>0</v>
@@ -5320,7 +5439,7 @@
         <v>35</v>
       </c>
       <c r="B12" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C12" s="51">
         <v>0</v>
@@ -5358,7 +5477,7 @@
         <v>36</v>
       </c>
       <c r="B13" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C13" s="51">
         <v>0</v>
@@ -5396,7 +5515,7 @@
         <v>37</v>
       </c>
       <c r="B14" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C14" s="51">
         <v>0</v>
@@ -5434,7 +5553,7 @@
         <v>38</v>
       </c>
       <c r="B15" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C15" s="51">
         <v>0</v>
@@ -5472,7 +5591,7 @@
         <v>39</v>
       </c>
       <c r="B16" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C16" s="51">
         <v>0</v>
@@ -5510,7 +5629,7 @@
         <v>40</v>
       </c>
       <c r="B17" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C17" s="51">
         <v>0</v>
@@ -5548,7 +5667,7 @@
         <v>41</v>
       </c>
       <c r="B18" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C18" s="51">
         <v>0</v>
@@ -5586,7 +5705,7 @@
         <v>42</v>
       </c>
       <c r="B19" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C19" s="51">
         <v>0</v>
@@ -5624,7 +5743,7 @@
         <v>43</v>
       </c>
       <c r="B20" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C20" s="51">
         <v>0</v>
@@ -5662,7 +5781,7 @@
         <v>44</v>
       </c>
       <c r="B21" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C21" s="51">
         <v>0</v>
@@ -5700,7 +5819,7 @@
         <v>45</v>
       </c>
       <c r="B22" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C22" s="51">
         <v>0</v>
@@ -5738,7 +5857,7 @@
         <v>46</v>
       </c>
       <c r="B23" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C23" s="51">
         <v>0</v>
@@ -5776,7 +5895,7 @@
         <v>47</v>
       </c>
       <c r="B24" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C24" s="51">
         <v>0</v>
@@ -5814,7 +5933,7 @@
         <v>48</v>
       </c>
       <c r="B25" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C25" s="51">
         <v>0</v>
@@ -5852,7 +5971,7 @@
         <v>49</v>
       </c>
       <c r="B26" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C26" s="51">
         <v>0</v>
@@ -5890,7 +6009,7 @@
         <v>50</v>
       </c>
       <c r="B27" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C27" s="51">
         <v>0</v>
@@ -5928,7 +6047,7 @@
         <v>51</v>
       </c>
       <c r="B28" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C28" s="51">
         <v>0</v>
@@ -5966,7 +6085,7 @@
         <v>52</v>
       </c>
       <c r="B29" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C29" s="51">
         <v>0</v>
@@ -6004,7 +6123,7 @@
         <v>53</v>
       </c>
       <c r="B30" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C30" s="51">
         <v>0</v>
@@ -6042,7 +6161,7 @@
         <v>54</v>
       </c>
       <c r="B31" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C31" s="51">
         <v>0</v>
@@ -6080,7 +6199,7 @@
         <v>55</v>
       </c>
       <c r="B32" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C32" s="51">
         <v>0</v>
@@ -6118,7 +6237,7 @@
         <v>56</v>
       </c>
       <c r="B33" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C33" s="51">
         <v>0.01</v>
@@ -6156,7 +6275,7 @@
         <v>57</v>
       </c>
       <c r="B34" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C34" s="51">
         <v>0.01</v>
@@ -6194,7 +6313,7 @@
         <v>58</v>
       </c>
       <c r="B35" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C35" s="51">
         <v>0.01</v>
@@ -6232,7 +6351,7 @@
         <v>59</v>
       </c>
       <c r="B36" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C36" s="51">
         <v>0.01</v>
@@ -6270,7 +6389,7 @@
         <v>60</v>
       </c>
       <c r="B37" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C37" s="51">
         <v>0.01</v>
@@ -6308,7 +6427,7 @@
         <v>61</v>
       </c>
       <c r="B38" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C38" s="51">
         <v>0.01</v>
@@ -6346,7 +6465,7 @@
         <v>62</v>
       </c>
       <c r="B39" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C39" s="51">
         <v>0.01</v>
@@ -6384,7 +6503,7 @@
         <v>63</v>
       </c>
       <c r="B40" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C40" s="51">
         <v>0.01</v>
@@ -6422,7 +6541,7 @@
         <v>64</v>
       </c>
       <c r="B41" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C41" s="51">
         <v>0.01</v>
@@ -6460,7 +6579,7 @@
         <v>65</v>
       </c>
       <c r="B42" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C42" s="51">
         <v>0.01</v>
@@ -6498,7 +6617,7 @@
         <v>66</v>
       </c>
       <c r="B43" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C43" s="51">
         <v>0.01</v>
@@ -6536,7 +6655,7 @@
         <v>67</v>
       </c>
       <c r="B44" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C44" s="51">
         <v>0.01</v>
@@ -6574,7 +6693,7 @@
         <v>68</v>
       </c>
       <c r="B45" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C45" s="51">
         <v>0.02</v>
@@ -6612,7 +6731,7 @@
         <v>69</v>
       </c>
       <c r="B46" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C46" s="51">
         <v>0.02</v>
@@ -6650,7 +6769,7 @@
         <v>70</v>
       </c>
       <c r="B47" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C47" s="51">
         <v>0.02</v>
@@ -6688,7 +6807,7 @@
         <v>71</v>
       </c>
       <c r="B48" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C48" s="51">
         <v>0.02</v>
@@ -6726,7 +6845,7 @@
         <v>72</v>
       </c>
       <c r="B49" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C49" s="51">
         <v>0.02</v>
@@ -6764,7 +6883,7 @@
         <v>73</v>
       </c>
       <c r="B50" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C50" s="51">
         <v>0.02</v>
@@ -6802,7 +6921,7 @@
         <v>74</v>
       </c>
       <c r="B51" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C51" s="51">
         <v>0.03</v>
@@ -6840,7 +6959,7 @@
         <v>75</v>
       </c>
       <c r="B52" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C52" s="51">
         <v>0.03</v>
@@ -6878,7 +6997,7 @@
         <v>76</v>
       </c>
       <c r="B53" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C53" s="51">
         <v>0.03</v>
@@ -6916,7 +7035,7 @@
         <v>77</v>
       </c>
       <c r="B54" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C54" s="51">
         <v>0.04</v>
@@ -6954,7 +7073,7 @@
         <v>78</v>
       </c>
       <c r="B55" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C55" s="51">
         <v>0.04</v>
@@ -6992,7 +7111,7 @@
         <v>79</v>
       </c>
       <c r="B56" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C56" s="51">
         <v>0.05</v>
@@ -7030,7 +7149,7 @@
         <v>80</v>
       </c>
       <c r="B57" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C57" s="51">
         <v>0.05</v>
@@ -7068,7 +7187,7 @@
         <v>81</v>
       </c>
       <c r="B58" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C58" s="51">
         <v>0.06</v>
@@ -7106,7 +7225,7 @@
         <v>82</v>
       </c>
       <c r="B59" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C59" s="51">
         <v>7.0000000000000007E-2</v>
@@ -7144,7 +7263,7 @@
         <v>83</v>
       </c>
       <c r="B60" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C60" s="51">
         <v>7.0000000000000007E-2</v>
@@ -7182,7 +7301,7 @@
         <v>84</v>
       </c>
       <c r="B61" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C61" s="51">
         <v>0.08</v>
@@ -7220,7 +7339,7 @@
         <v>85</v>
       </c>
       <c r="B62" s="51" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C62" s="51">
         <v>0.09</v>
@@ -7258,7 +7377,7 @@
         <v>25</v>
       </c>
       <c r="B63" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C63" s="51">
         <v>0</v>
@@ -7296,7 +7415,7 @@
         <v>26</v>
       </c>
       <c r="B64" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C64" s="51">
         <v>0</v>
@@ -7334,7 +7453,7 @@
         <v>27</v>
       </c>
       <c r="B65" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C65" s="51">
         <v>0</v>
@@ -7372,7 +7491,7 @@
         <v>28</v>
       </c>
       <c r="B66" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C66" s="51">
         <v>0</v>
@@ -7410,7 +7529,7 @@
         <v>29</v>
       </c>
       <c r="B67" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C67" s="51">
         <v>0</v>
@@ -7448,7 +7567,7 @@
         <v>30</v>
       </c>
       <c r="B68" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C68" s="51">
         <v>0</v>
@@ -7486,7 +7605,7 @@
         <v>31</v>
       </c>
       <c r="B69" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C69" s="51">
         <v>0</v>
@@ -7524,7 +7643,7 @@
         <v>32</v>
       </c>
       <c r="B70" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C70" s="51">
         <v>0</v>
@@ -7562,7 +7681,7 @@
         <v>33</v>
       </c>
       <c r="B71" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C71" s="51">
         <v>0</v>
@@ -7600,7 +7719,7 @@
         <v>34</v>
       </c>
       <c r="B72" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C72" s="51">
         <v>0</v>
@@ -7638,7 +7757,7 @@
         <v>35</v>
       </c>
       <c r="B73" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C73" s="51">
         <v>0</v>
@@ -7676,7 +7795,7 @@
         <v>36</v>
       </c>
       <c r="B74" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C74" s="51">
         <v>0</v>
@@ -7714,7 +7833,7 @@
         <v>37</v>
       </c>
       <c r="B75" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C75" s="51">
         <v>0</v>
@@ -7752,7 +7871,7 @@
         <v>38</v>
       </c>
       <c r="B76" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C76" s="51">
         <v>0</v>
@@ -7790,7 +7909,7 @@
         <v>39</v>
       </c>
       <c r="B77" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C77" s="51">
         <v>0</v>
@@ -7828,7 +7947,7 @@
         <v>40</v>
       </c>
       <c r="B78" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C78" s="51">
         <v>0</v>
@@ -7866,7 +7985,7 @@
         <v>41</v>
       </c>
       <c r="B79" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C79" s="51">
         <v>0</v>
@@ -7904,7 +8023,7 @@
         <v>42</v>
       </c>
       <c r="B80" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C80" s="51">
         <v>0</v>
@@ -7942,7 +8061,7 @@
         <v>43</v>
       </c>
       <c r="B81" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C81" s="51">
         <v>0</v>
@@ -7980,7 +8099,7 @@
         <v>44</v>
       </c>
       <c r="B82" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C82" s="51">
         <v>0</v>
@@ -8018,7 +8137,7 @@
         <v>45</v>
       </c>
       <c r="B83" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C83" s="51">
         <v>0</v>
@@ -8056,7 +8175,7 @@
         <v>46</v>
       </c>
       <c r="B84" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C84" s="51">
         <v>0</v>
@@ -8094,7 +8213,7 @@
         <v>47</v>
       </c>
       <c r="B85" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C85" s="51">
         <v>0</v>
@@ -8132,7 +8251,7 @@
         <v>48</v>
       </c>
       <c r="B86" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C86" s="51">
         <v>0</v>
@@ -8170,7 +8289,7 @@
         <v>49</v>
       </c>
       <c r="B87" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C87" s="51">
         <v>0</v>
@@ -8208,7 +8327,7 @@
         <v>50</v>
       </c>
       <c r="B88" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C88" s="51">
         <v>0</v>
@@ -8246,7 +8365,7 @@
         <v>51</v>
       </c>
       <c r="B89" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C89" s="51">
         <v>0</v>
@@ -8284,7 +8403,7 @@
         <v>52</v>
       </c>
       <c r="B90" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C90" s="51">
         <v>0</v>
@@ -8322,7 +8441,7 @@
         <v>53</v>
       </c>
       <c r="B91" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C91" s="51">
         <v>0</v>
@@ -8360,7 +8479,7 @@
         <v>54</v>
       </c>
       <c r="B92" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C92" s="51">
         <v>0</v>
@@ -8398,7 +8517,7 @@
         <v>55</v>
       </c>
       <c r="B93" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C93" s="51">
         <v>0</v>
@@ -8436,7 +8555,7 @@
         <v>56</v>
       </c>
       <c r="B94" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C94" s="51">
         <v>0</v>
@@ -8474,7 +8593,7 @@
         <v>57</v>
       </c>
       <c r="B95" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C95" s="51">
         <v>0</v>
@@ -8512,7 +8631,7 @@
         <v>58</v>
       </c>
       <c r="B96" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C96" s="51">
         <v>0</v>
@@ -8550,7 +8669,7 @@
         <v>59</v>
       </c>
       <c r="B97" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C97" s="51">
         <v>0</v>
@@ -8588,7 +8707,7 @@
         <v>60</v>
       </c>
       <c r="B98" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C98" s="51">
         <v>0</v>
@@ -8626,7 +8745,7 @@
         <v>61</v>
       </c>
       <c r="B99" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C99" s="51">
         <v>0.01</v>
@@ -8664,7 +8783,7 @@
         <v>62</v>
       </c>
       <c r="B100" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C100" s="51">
         <v>0.01</v>
@@ -8702,7 +8821,7 @@
         <v>63</v>
       </c>
       <c r="B101" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C101" s="51">
         <v>0.01</v>
@@ -8740,7 +8859,7 @@
         <v>64</v>
       </c>
       <c r="B102" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C102" s="51">
         <v>0.01</v>
@@ -8778,7 +8897,7 @@
         <v>65</v>
       </c>
       <c r="B103" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C103" s="51">
         <v>0.01</v>
@@ -8816,7 +8935,7 @@
         <v>66</v>
       </c>
       <c r="B104" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C104" s="51">
         <v>0.01</v>
@@ -8854,7 +8973,7 @@
         <v>67</v>
       </c>
       <c r="B105" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C105" s="51">
         <v>0.01</v>
@@ -8892,7 +9011,7 @@
         <v>68</v>
       </c>
       <c r="B106" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C106" s="51">
         <v>0.01</v>
@@ -8930,7 +9049,7 @@
         <v>69</v>
       </c>
       <c r="B107" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C107" s="51">
         <v>0.01</v>
@@ -8968,7 +9087,7 @@
         <v>70</v>
       </c>
       <c r="B108" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C108" s="51">
         <v>0.01</v>
@@ -9006,7 +9125,7 @@
         <v>71</v>
       </c>
       <c r="B109" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C109" s="51">
         <v>0.01</v>
@@ -9044,7 +9163,7 @@
         <v>72</v>
       </c>
       <c r="B110" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C110" s="51">
         <v>0.01</v>
@@ -9082,7 +9201,7 @@
         <v>73</v>
       </c>
       <c r="B111" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C111" s="51">
         <v>0.02</v>
@@ -9120,7 +9239,7 @@
         <v>74</v>
       </c>
       <c r="B112" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C112" s="51">
         <v>0.02</v>
@@ -9158,7 +9277,7 @@
         <v>75</v>
       </c>
       <c r="B113" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C113" s="51">
         <v>0.02</v>
@@ -9196,7 +9315,7 @@
         <v>76</v>
       </c>
       <c r="B114" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C114" s="51">
         <v>0.02</v>
@@ -9234,7 +9353,7 @@
         <v>77</v>
       </c>
       <c r="B115" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C115" s="51">
         <v>0.03</v>
@@ -9272,7 +9391,7 @@
         <v>78</v>
       </c>
       <c r="B116" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C116" s="51">
         <v>0.03</v>
@@ -9310,7 +9429,7 @@
         <v>79</v>
       </c>
       <c r="B117" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C117" s="51">
         <v>0.03</v>
@@ -9348,7 +9467,7 @@
         <v>80</v>
       </c>
       <c r="B118" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C118" s="51">
         <v>0.04</v>
@@ -9386,7 +9505,7 @@
         <v>81</v>
       </c>
       <c r="B119" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C119" s="51">
         <v>0.04</v>
@@ -9424,7 +9543,7 @@
         <v>82</v>
       </c>
       <c r="B120" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C120" s="51">
         <v>0.05</v>
@@ -9462,7 +9581,7 @@
         <v>83</v>
       </c>
       <c r="B121" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C121" s="51">
         <v>0.05</v>
@@ -9500,7 +9619,7 @@
         <v>84</v>
       </c>
       <c r="B122" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C122" s="51">
         <v>0.06</v>
@@ -9538,7 +9657,7 @@
         <v>85</v>
       </c>
       <c r="B123" s="51" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C123" s="51">
         <v>7.0000000000000007E-2</v>

</xml_diff>

<commit_message>
KCP-77 - wip, look at UI transforms
</commit_message>
<xml_diff>
--- a/resources/kcp-models-master.xlsx
+++ b/resources/kcp-models-master.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28122"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{70E85B90-2538-4DE0-8EDA-C110139F2379}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5B3CED99-68A8-4EDB-973B-6A58D5EE0448}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080" firstSheet="6" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="125">
   <si>
     <t>Notes</t>
   </si>
@@ -474,7 +474,7 @@
     <t>Age at surgery</t>
   </si>
   <si>
-    <t>:numeric</t>
+    <t>{:dps 1, :max 85, :min 25, :type :numeric}</t>
   </si>
   <si>
     <t>Age when the kidney cancer surgery was performed. An age between 25 and 85 may be entered here.</t>
@@ -483,7 +483,7 @@
     <t>:sex</t>
   </si>
   <si>
-    <t>:male</t>
+    <t>:Male</t>
   </si>
   <si>
     <t>Sex</t>
@@ -492,7 +492,7 @@
     <t>Male</t>
   </si>
   <si>
-    <t>:female</t>
+    <t>:Female</t>
   </si>
   <si>
     <t>Female</t>
@@ -772,7 +772,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -857,6 +857,8 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4229,7 +4231,7 @@
       <c r="D2" s="42" t="s">
         <v>46</v>
       </c>
-      <c r="E2" s="43">
+      <c r="E2" s="52">
         <v>0</v>
       </c>
       <c r="F2" s="42" t="s">
@@ -4265,7 +4267,7 @@
       <c r="D3" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="E3" s="25">
+      <c r="E3" s="53">
         <v>1.2430000000000001</v>
       </c>
       <c r="F3" s="4"/>
@@ -4296,7 +4298,7 @@
       <c r="D4" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="E4" s="25">
+      <c r="E4" s="53">
         <v>1.6479999999999999</v>
       </c>
       <c r="F4" s="4"/>
@@ -4327,7 +4329,7 @@
       <c r="D5" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="E5" s="25">
+      <c r="E5" s="53">
         <v>1.6479999999999999</v>
       </c>
       <c r="F5" s="4"/>
@@ -4358,7 +4360,7 @@
       <c r="D6" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="E6" s="25">
+      <c r="E6" s="53">
         <v>1.8959999999999999</v>
       </c>
       <c r="F6" s="4"/>
@@ -4389,7 +4391,7 @@
       <c r="D7" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="E7" s="25">
+      <c r="E7" s="53">
         <v>2.0139999999999998</v>
       </c>
       <c r="F7" s="4"/>
@@ -4420,7 +4422,7 @@
       <c r="D8" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="E8" s="25">
+      <c r="E8" s="53">
         <v>2.0139999999999998</v>
       </c>
       <c r="F8" s="4"/>
@@ -4451,7 +4453,7 @@
       <c r="D9" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="E9" s="25">
+      <c r="E9" s="53">
         <v>2.0139999999999998</v>
       </c>
       <c r="F9" s="4"/>
@@ -4477,7 +4479,7 @@
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
+      <c r="E10" s="53"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="46"/>
@@ -4501,7 +4503,7 @@
       <c r="D11" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="E11" s="25">
+      <c r="E11" s="53">
         <v>0</v>
       </c>
       <c r="F11" s="9" t="s">
@@ -4537,7 +4539,7 @@
       <c r="D12" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="E12" s="25">
+      <c r="E12" s="53">
         <v>0</v>
       </c>
       <c r="F12" s="9" t="s">
@@ -4571,7 +4573,7 @@
       <c r="D13" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="E13" s="25">
+      <c r="E13" s="53">
         <v>0.92400000000000004</v>
       </c>
       <c r="F13" s="9" t="s">
@@ -4599,7 +4601,7 @@
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
+      <c r="E14" s="53"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="46"/>
@@ -4623,7 +4625,7 @@
       <c r="D15" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="E15" s="25">
+      <c r="E15" s="53">
         <v>0</v>
       </c>
       <c r="F15" s="9" t="s">
@@ -4657,7 +4659,7 @@
       <c r="D16" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="E16" s="25">
+      <c r="E16" s="53">
         <v>0.39300000000000002</v>
       </c>
       <c r="F16" s="9" t="s">
@@ -4683,7 +4685,7 @@
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
+      <c r="E17" s="53"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="46"/>
@@ -4707,7 +4709,7 @@
       <c r="D18" s="25">
         <v>1</v>
       </c>
-      <c r="E18" s="25">
+      <c r="E18" s="53">
         <v>0</v>
       </c>
       <c r="F18" s="9" t="s">
@@ -4741,7 +4743,7 @@
       <c r="D19" s="25">
         <v>2</v>
       </c>
-      <c r="E19" s="25">
+      <c r="E19" s="53">
         <v>0</v>
       </c>
       <c r="F19" s="9" t="s">
@@ -4773,7 +4775,7 @@
       <c r="D20" s="25">
         <v>3</v>
       </c>
-      <c r="E20" s="25">
+      <c r="E20" s="53">
         <v>0.64</v>
       </c>
       <c r="F20" s="9" t="s">
@@ -4805,7 +4807,7 @@
       <c r="D21" s="25">
         <v>4</v>
       </c>
-      <c r="E21" s="25">
+      <c r="E21" s="53">
         <v>1.3129999999999999</v>
       </c>
       <c r="F21" s="9" t="s">
@@ -4831,7 +4833,7 @@
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
       <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
+      <c r="E22" s="53"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="46"/>
@@ -4855,7 +4857,7 @@
       <c r="D23" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="E23" s="25">
+      <c r="E23" s="53">
         <v>0</v>
       </c>
       <c r="F23" s="9" t="s">
@@ -4889,7 +4891,7 @@
       <c r="D24" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="E24" s="25">
+      <c r="E24" s="53">
         <v>0.67800000000000005</v>
       </c>
       <c r="F24" s="9" t="s">
@@ -4919,7 +4921,7 @@
         <v>103</v>
       </c>
       <c r="D25" s="9"/>
-      <c r="E25" s="25"/>
+      <c r="E25" s="53"/>
       <c r="F25" s="9" t="s">
         <v>104</v>
       </c>
@@ -4951,7 +4953,9 @@
       <c r="D26" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="E26" s="25"/>
+      <c r="E26" s="53">
+        <v>0</v>
+      </c>
       <c r="F26" s="9" t="s">
         <v>47</v>
       </c>
@@ -4977,13 +4981,13 @@
       <c r="B27" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="C27" s="9" t="s">
-        <v>108</v>
-      </c>
+      <c r="C27" s="9"/>
       <c r="D27" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="E27" s="25"/>
+      <c r="E27" s="53">
+        <v>0</v>
+      </c>
       <c r="F27" s="9" t="s">
         <v>47</v>
       </c>

</xml_diff>

<commit_message>
KCP-90 - update printout based on feedback
</commit_message>
<xml_diff>
--- a/resources/kcp-models-master.xlsx
+++ b/resources/kcp-models-master.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28318"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28409"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D9D096E1-1831-45A5-8C56-572661716DA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F150EB0C-282B-4FF8-9A48-0C23826D5C03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -201,7 +201,7 @@
   </si>
   <si>
     <t>[:div "The pathological stage of a kidney cancer tumour is a measure of its size and how far it has spread. This is determined by assessing cancer tissue removed during surgery."
-   [:ul
+   [:ul { :class-name "more-info-list" }
       [:li "Stage 1a (or pT1a) – the cancer is small (4cm or smaller) and only inside the kidney"]
       [:li "Stage 1b (or pT1b) – the cancer is small (between 4cm and 7 cm) and only inside the kidney"]
       [:li "Stage 2a (pT2a) - the cancer is between 7cm and 10cm and only inside the kidney"]
@@ -288,8 +288,8 @@
     <t>there were no lymph nodes found in the tumour samples removed at the time of surgery</t>
   </si>
   <si>
-    <t>[:div "The regional lymph node status indicates if the cancer has spread to lymph nodes near the kidney. Lymph nodes are a network of glands found throughout the body that drain away waste products and fight infections. Lymph nodes near the kidney may be removed during surgery and tested for the presence of cancer."   
-    [:ul
+    <t>[:div "The regional lymph node status indicates if the cancer has spread to lymph nodes near the kidney. Lymph nodes are a network of glands found throughout the body that drain away waste products and fight infections. Lymph nodes near the kidney may be removed during surgery and tested for the presence of cancer.  However, it is common for no lymph nodes to be removed at the time of surgery and no further investigation to be required."
+    [:ul  { :class-name "more-info-list" }
         [:li "No investigation required (pNx) - There were no lymph nodes in the tissue removed at surgery. This is common if there are no noticeable lymph nodes present."]
         [:li "pN0 – No cancer was detected in any lymph nodes near the tumour."]
         [:li "pN1 – Cancer cells were detected in one or more lymph nodes near the tumour."]]

</xml_diff>

<commit_message>
KCP-99 - update configure step to include new spreadsheet entries and tool
</commit_message>
<xml_diff>
--- a/resources/kcp-models-master.xlsx
+++ b/resources/kcp-models-master.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\kcp2\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6675DE73-B5EB-4C30-B086-82ADE3F8FFC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{546D93B7-7C2D-4E7C-9D5C-A33B537C3C00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -14033,7 +14033,7 @@
         <v>30</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C3" s="4"/>
       <c r="D3" s="9" t="s">
@@ -14064,7 +14064,7 @@
         <v>30</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C4" s="4"/>
       <c r="D4" s="9" t="s">
@@ -14095,7 +14095,7 @@
         <v>30</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="C5" s="4"/>
       <c r="D5" s="9" t="s">

</xml_diff>

<commit_message>
KCP-105 - printout handling for ccs & alternate risk statements
</commit_message>
<xml_diff>
--- a/resources/kcp-models-master.xlsx
+++ b/resources/kcp-models-master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\kcp\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B56A9581-4766-4D3C-9198-22122D9BB762}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40964FC5-6DA5-4991-B335-CA27030D669A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1560" yWindow="1560" windowWidth="38700" windowHeight="15285" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -689,12 +689,6 @@
     </r>
   </si>
   <si>
-    <t>[:div
-  [:p "The Charlson Comorbidity Score is a measure of the number and severity of long-term conditions present for an individual. It includes 15 conditions in addition to cancer. Details of how this calculated can be found in the technical section."]
-  [:p "A high Charlson Score indicates that a patient is frail and less likely to benefit from further treatment for kidney cancer."]
-]</t>
-  </si>
-  <si>
     <t>[:p "Age when the kidney cancer surgery was performed. Older patients are more at risk of other long-term health conditions and are relatively less likely to die from kidney cancer. An age between 25 and 85 may be entered here."]</t>
   </si>
   <si>
@@ -702,6 +696,11 @@
   </si>
   <si>
     <t>{:dps 0, :max 31, :min 2, :type :numeric :validation "Score must be between 2 and 31"  :calc-workflow :charlson}</t>
+  </si>
+  <si>
+    <t>[:p [:span "The Charlson Comorbidity Score is a measure of the number and severity of long-term conditions present for an individual."
+[:span {:class-name "d-print-none" } " It includes 15 conditions in addition to cancer. Details of how this calculated can be found in the technical section."]
+" A high Charlson Score indicates that a patient is frail and less likely to benefit from further treatment for kidney cancer."]]</t>
   </si>
   <si>
     <t>Never used tobacco</t>
@@ -9079,11 +9078,11 @@
       <c r="D25" s="9"/>
       <c r="E25" s="53"/>
       <c r="F25" s="9" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="G25" s="4"/>
       <c r="H25" s="49" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I25" s="25">
         <v>100</v>
@@ -14630,11 +14629,11 @@
       <c r="D21" s="9"/>
       <c r="E21" s="53"/>
       <c r="F21" s="9" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="G21" s="4"/>
       <c r="H21" s="49" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I21" s="25">
         <v>100</v>
@@ -14724,11 +14723,11 @@
       <c r="D24" s="9"/>
       <c r="E24" s="53"/>
       <c r="F24" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G24" s="4"/>
       <c r="H24" s="49" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="I24" s="25">
         <v>120</v>

</xml_diff>

<commit_message>
KCP-101 - input updates
</commit_message>
<xml_diff>
--- a/resources/kcp-models-master.xlsx
+++ b/resources/kcp-models-master.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\kcp2\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{546D93B7-7C2D-4E7C-9D5C-A33B537C3C00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{217B294A-7196-43DD-95BD-C45F3F20F84B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="151">
   <si>
     <t>Notes</t>
   </si>
@@ -505,9 +505,6 @@
     <t>{:dps 0, :max 85, :min 25, :type :numeric}</t>
   </si>
   <si>
-    <t>[:p "Age when the kidney cancer surgery was performed. An age between 25 and 85 may be entered here."]</t>
-  </si>
-  <si>
     <t>:Male</t>
   </si>
   <si>
@@ -563,15 +560,6 @@
   </si>
   <si>
     <t>1</t>
-  </si>
-  <si>
-    <t>[:div "The pathological stage of a kidney cancer tumour is a measure of its size and how far it has spread. This is determined by assessing cancer tissue removed during surgery. "
-   [:ul { :class-name "more-info-list" }
-      [:li "Stage 1 (or pT1) - the cancer is small (&lt;7cm) and only inside the kidney"]
-      [:li "Stage 2 (or pT2) - the cancer is larger (&gt;7cm) and only inside the kidney"]
-      [:li "Stage 3 (or pT3) - that cancer is growing into the area surrounding the kidney (this can include growing into the fat around the kidney, the renal vein or the vena cava)"]
-      [:li "Stage 4 (or pT4) - the cancer has spread through the capsule that surrounds the kidney. It may have grown into the adrenal gland."]]
-]</t>
   </si>
   <si>
     <t>2</t>
@@ -652,6 +640,71 @@
   </si>
   <si>
     <t>:Never</t>
+  </si>
+  <si>
+    <t>[:div "The pathological stage of a kidney cancer tumour is a measure of its size and how far it has spread. This is determined by assessing cancer tissue removed during surgery. "
+   [:ul { :class-name "more-info-list" }
+      [:li "Stage 1 (or pT1) - the cancer is small (&lt;7cm) and only inside the kidney"]
+      [:li "Stage 2 (or pT2) - the cancer is larger (&gt;7cm) and only inside the kidney"]
+      [:li "Stage 3 (or pT3) - that cancer is growing into the area surrounding the kidney (this can include growing into the fat around the kidney, the renal vein or the vena cava)"]
+      [:li "Stage 4 (or pT4) - the cancer has spread through the capsule that surrounds the kidney. It may have grown into the adrenal gland."]]
+   "The model does not differentiate between stage sub-classifications (such as T2a or T2b)."
+]</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">[:p </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+      </rPr>
+      <t>"The size of the kidney cancer tumour removed during surgery. This factor is not used in the PREDICT-Kidney model (and so will not affect the estimated risks). It is included in the tool as it used to calculate the Leibovich score and assess eligibility for adjuvant treatment."</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+      </rPr>
+      <t>]</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">[:p </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+      </rPr>
+      <t>"The tumour necrosis indicates if dead cancer cells were found in the samples removed at surgery. Dead cells may indicate a faster-growing tumour. If necrosis was detected the cancer is more likely to return. This factor is not used in the PREDICT-Kidney model (and so will not affect the estimated risks). It is included in the tool as it used to calculate the Leibovich score and assess eligibility for adjuvant treatment."</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+      </rPr>
+      <t>]</t>
+    </r>
+  </si>
+  <si>
+    <t>[:div
+  [:p "The Charlson Comorbidity Score is a measure of the number and severity of long-term conditions present for an individual. It includes 15 conditions in addition to cancer. Details of how this calculated can be found in the technical section."]
+  [:p "A high Charlson Score indicates that a patient is frail and less likely to benefit from further treatment for kidney cancer."]
+]</t>
+  </si>
+  <si>
+    <t>[:p "Age when the kidney cancer surgery was performed. Older patients are more at risk of other long-term health conditions and are relatively less likely to die from kidney cancer. An age between 25 and 85 may be entered here."]</t>
   </si>
 </sst>
 </file>
@@ -2261,13 +2314,13 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
+        <v>138</v>
+      </c>
+      <c r="B1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C1" t="s">
         <v>140</v>
-      </c>
-      <c r="B1" t="s">
-        <v>141</v>
-      </c>
-      <c r="C1" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -2289,7 +2342,7 @@
         <v>0.42</v>
       </c>
       <c r="C3" s="54" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -4229,13 +4282,13 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
+        <v>138</v>
+      </c>
+      <c r="B1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C1" t="s">
         <v>140</v>
-      </c>
-      <c r="B1" t="s">
-        <v>141</v>
-      </c>
-      <c r="C1" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -6362,7 +6415,7 @@
     </row>
     <row r="3" spans="1:5" ht="17.100000000000001" customHeight="1">
       <c r="A3" s="23" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B3" s="21" t="s">
         <v>19</v>
@@ -9023,7 +9076,7 @@
       </c>
       <c r="G25" s="4"/>
       <c r="H25" s="49" t="s">
-        <v>107</v>
+        <v>150</v>
       </c>
       <c r="I25" s="25">
         <v>100</v>
@@ -9041,13 +9094,13 @@
         <v>34</v>
       </c>
       <c r="B26" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="C26" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="D26" s="9" t="s">
         <v>109</v>
-      </c>
-      <c r="D26" s="9" t="s">
-        <v>110</v>
       </c>
       <c r="E26" s="53">
         <v>0</v>
@@ -9063,7 +9116,7 @@
       <c r="J26" s="4"/>
       <c r="K26" s="4"/>
       <c r="L26" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="M26" s="4"/>
       <c r="N26" s="44">
@@ -9075,11 +9128,11 @@
         <v>34</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C27" s="9"/>
       <c r="D27" s="9" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E27" s="53">
         <v>0</v>
@@ -9095,7 +9148,7 @@
       <c r="J27" s="4"/>
       <c r="K27" s="4"/>
       <c r="L27" s="9" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="M27" s="4"/>
       <c r="N27" s="44">
@@ -9118,40 +9171,40 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="50" t="s">
+        <v>112</v>
+      </c>
+      <c r="B1" s="50" t="s">
+        <v>108</v>
+      </c>
+      <c r="C1" s="50" t="s">
         <v>113</v>
       </c>
-      <c r="B1" s="50" t="s">
-        <v>109</v>
-      </c>
-      <c r="C1" s="50" t="s">
+      <c r="D1" s="50" t="s">
         <v>114</v>
       </c>
-      <c r="D1" s="50" t="s">
+      <c r="E1" s="50" t="s">
         <v>115</v>
       </c>
-      <c r="E1" s="50" t="s">
+      <c r="F1" s="50" t="s">
         <v>116</v>
       </c>
-      <c r="F1" s="50" t="s">
+      <c r="G1" s="50" t="s">
         <v>117</v>
       </c>
-      <c r="G1" s="50" t="s">
+      <c r="H1" s="50" t="s">
         <v>118</v>
       </c>
-      <c r="H1" s="50" t="s">
+      <c r="I1" s="50" t="s">
         <v>119</v>
       </c>
-      <c r="I1" s="50" t="s">
+      <c r="J1" s="50" t="s">
         <v>120</v>
       </c>
-      <c r="J1" s="50" t="s">
+      <c r="K1" s="50" t="s">
         <v>121</v>
       </c>
-      <c r="K1" s="50" t="s">
+      <c r="L1" s="50" t="s">
         <v>122</v>
-      </c>
-      <c r="L1" s="50" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:12">
@@ -9159,7 +9212,7 @@
         <v>25</v>
       </c>
       <c r="B2" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C2" s="51">
         <v>0</v>
@@ -9197,7 +9250,7 @@
         <v>26</v>
       </c>
       <c r="B3" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C3" s="51">
         <v>0</v>
@@ -9235,7 +9288,7 @@
         <v>27</v>
       </c>
       <c r="B4" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C4" s="51">
         <v>0</v>
@@ -9273,7 +9326,7 @@
         <v>28</v>
       </c>
       <c r="B5" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C5" s="51">
         <v>0</v>
@@ -9311,7 +9364,7 @@
         <v>29</v>
       </c>
       <c r="B6" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C6" s="51">
         <v>0</v>
@@ -9349,7 +9402,7 @@
         <v>30</v>
       </c>
       <c r="B7" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C7" s="51">
         <v>0</v>
@@ -9387,7 +9440,7 @@
         <v>31</v>
       </c>
       <c r="B8" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C8" s="51">
         <v>0</v>
@@ -9425,7 +9478,7 @@
         <v>32</v>
       </c>
       <c r="B9" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C9" s="51">
         <v>0</v>
@@ -9463,7 +9516,7 @@
         <v>33</v>
       </c>
       <c r="B10" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C10" s="51">
         <v>0</v>
@@ -9501,7 +9554,7 @@
         <v>34</v>
       </c>
       <c r="B11" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C11" s="51">
         <v>0</v>
@@ -9539,7 +9592,7 @@
         <v>35</v>
       </c>
       <c r="B12" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C12" s="51">
         <v>0</v>
@@ -9577,7 +9630,7 @@
         <v>36</v>
       </c>
       <c r="B13" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C13" s="51">
         <v>0</v>
@@ -9615,7 +9668,7 @@
         <v>37</v>
       </c>
       <c r="B14" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C14" s="51">
         <v>0</v>
@@ -9653,7 +9706,7 @@
         <v>38</v>
       </c>
       <c r="B15" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C15" s="51">
         <v>0</v>
@@ -9691,7 +9744,7 @@
         <v>39</v>
       </c>
       <c r="B16" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C16" s="51">
         <v>0</v>
@@ -9729,7 +9782,7 @@
         <v>40</v>
       </c>
       <c r="B17" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C17" s="51">
         <v>0</v>
@@ -9767,7 +9820,7 @@
         <v>41</v>
       </c>
       <c r="B18" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C18" s="51">
         <v>0</v>
@@ -9805,7 +9858,7 @@
         <v>42</v>
       </c>
       <c r="B19" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C19" s="51">
         <v>0</v>
@@ -9843,7 +9896,7 @@
         <v>43</v>
       </c>
       <c r="B20" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C20" s="51">
         <v>0</v>
@@ -9881,7 +9934,7 @@
         <v>44</v>
       </c>
       <c r="B21" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C21" s="51">
         <v>0</v>
@@ -9919,7 +9972,7 @@
         <v>45</v>
       </c>
       <c r="B22" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C22" s="51">
         <v>0</v>
@@ -9957,7 +10010,7 @@
         <v>46</v>
       </c>
       <c r="B23" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C23" s="51">
         <v>0</v>
@@ -9995,7 +10048,7 @@
         <v>47</v>
       </c>
       <c r="B24" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C24" s="51">
         <v>0</v>
@@ -10033,7 +10086,7 @@
         <v>48</v>
       </c>
       <c r="B25" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C25" s="51">
         <v>0</v>
@@ -10071,7 +10124,7 @@
         <v>49</v>
       </c>
       <c r="B26" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C26" s="51">
         <v>0</v>
@@ -10109,7 +10162,7 @@
         <v>50</v>
       </c>
       <c r="B27" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C27" s="51">
         <v>0</v>
@@ -10147,7 +10200,7 @@
         <v>51</v>
       </c>
       <c r="B28" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C28" s="51">
         <v>0</v>
@@ -10185,7 +10238,7 @@
         <v>52</v>
       </c>
       <c r="B29" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C29" s="51">
         <v>0</v>
@@ -10223,7 +10276,7 @@
         <v>53</v>
       </c>
       <c r="B30" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C30" s="51">
         <v>0</v>
@@ -10261,7 +10314,7 @@
         <v>54</v>
       </c>
       <c r="B31" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C31" s="51">
         <v>0</v>
@@ -10299,7 +10352,7 @@
         <v>55</v>
       </c>
       <c r="B32" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C32" s="51">
         <v>0</v>
@@ -10337,7 +10390,7 @@
         <v>56</v>
       </c>
       <c r="B33" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C33" s="51">
         <v>0.01</v>
@@ -10375,7 +10428,7 @@
         <v>57</v>
       </c>
       <c r="B34" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C34" s="51">
         <v>0.01</v>
@@ -10413,7 +10466,7 @@
         <v>58</v>
       </c>
       <c r="B35" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C35" s="51">
         <v>0.01</v>
@@ -10451,7 +10504,7 @@
         <v>59</v>
       </c>
       <c r="B36" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C36" s="51">
         <v>0.01</v>
@@ -10489,7 +10542,7 @@
         <v>60</v>
       </c>
       <c r="B37" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C37" s="51">
         <v>0.01</v>
@@ -10527,7 +10580,7 @@
         <v>61</v>
       </c>
       <c r="B38" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C38" s="51">
         <v>0.01</v>
@@ -10565,7 +10618,7 @@
         <v>62</v>
       </c>
       <c r="B39" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C39" s="51">
         <v>0.01</v>
@@ -10603,7 +10656,7 @@
         <v>63</v>
       </c>
       <c r="B40" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C40" s="51">
         <v>0.01</v>
@@ -10641,7 +10694,7 @@
         <v>64</v>
       </c>
       <c r="B41" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C41" s="51">
         <v>0.01</v>
@@ -10679,7 +10732,7 @@
         <v>65</v>
       </c>
       <c r="B42" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C42" s="51">
         <v>0.01</v>
@@ -10717,7 +10770,7 @@
         <v>66</v>
       </c>
       <c r="B43" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C43" s="51">
         <v>0.01</v>
@@ -10755,7 +10808,7 @@
         <v>67</v>
       </c>
       <c r="B44" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C44" s="51">
         <v>0.01</v>
@@ -10793,7 +10846,7 @@
         <v>68</v>
       </c>
       <c r="B45" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C45" s="51">
         <v>0.02</v>
@@ -10831,7 +10884,7 @@
         <v>69</v>
       </c>
       <c r="B46" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C46" s="51">
         <v>0.02</v>
@@ -10869,7 +10922,7 @@
         <v>70</v>
       </c>
       <c r="B47" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C47" s="51">
         <v>0.02</v>
@@ -10907,7 +10960,7 @@
         <v>71</v>
       </c>
       <c r="B48" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C48" s="51">
         <v>0.02</v>
@@ -10945,7 +10998,7 @@
         <v>72</v>
       </c>
       <c r="B49" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C49" s="51">
         <v>0.02</v>
@@ -10983,7 +11036,7 @@
         <v>73</v>
       </c>
       <c r="B50" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C50" s="51">
         <v>0.02</v>
@@ -11021,7 +11074,7 @@
         <v>74</v>
       </c>
       <c r="B51" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C51" s="51">
         <v>0.03</v>
@@ -11059,7 +11112,7 @@
         <v>75</v>
       </c>
       <c r="B52" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C52" s="51">
         <v>0.03</v>
@@ -11097,7 +11150,7 @@
         <v>76</v>
       </c>
       <c r="B53" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C53" s="51">
         <v>0.03</v>
@@ -11135,7 +11188,7 @@
         <v>77</v>
       </c>
       <c r="B54" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C54" s="51">
         <v>0.04</v>
@@ -11173,7 +11226,7 @@
         <v>78</v>
       </c>
       <c r="B55" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C55" s="51">
         <v>0.04</v>
@@ -11211,7 +11264,7 @@
         <v>79</v>
       </c>
       <c r="B56" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C56" s="51">
         <v>0.05</v>
@@ -11249,7 +11302,7 @@
         <v>80</v>
       </c>
       <c r="B57" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C57" s="51">
         <v>0.05</v>
@@ -11287,7 +11340,7 @@
         <v>81</v>
       </c>
       <c r="B58" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C58" s="51">
         <v>0.06</v>
@@ -11325,7 +11378,7 @@
         <v>82</v>
       </c>
       <c r="B59" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C59" s="51">
         <v>7.0000000000000007E-2</v>
@@ -11363,7 +11416,7 @@
         <v>83</v>
       </c>
       <c r="B60" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C60" s="51">
         <v>7.0000000000000007E-2</v>
@@ -11401,7 +11454,7 @@
         <v>84</v>
       </c>
       <c r="B61" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C61" s="51">
         <v>0.08</v>
@@ -11439,7 +11492,7 @@
         <v>85</v>
       </c>
       <c r="B62" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C62" s="51">
         <v>0.09</v>
@@ -11477,7 +11530,7 @@
         <v>25</v>
       </c>
       <c r="B63" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C63" s="51">
         <v>0</v>
@@ -11515,7 +11568,7 @@
         <v>26</v>
       </c>
       <c r="B64" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C64" s="51">
         <v>0</v>
@@ -11553,7 +11606,7 @@
         <v>27</v>
       </c>
       <c r="B65" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C65" s="51">
         <v>0</v>
@@ -11591,7 +11644,7 @@
         <v>28</v>
       </c>
       <c r="B66" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C66" s="51">
         <v>0</v>
@@ -11629,7 +11682,7 @@
         <v>29</v>
       </c>
       <c r="B67" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C67" s="51">
         <v>0</v>
@@ -11667,7 +11720,7 @@
         <v>30</v>
       </c>
       <c r="B68" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C68" s="51">
         <v>0</v>
@@ -11705,7 +11758,7 @@
         <v>31</v>
       </c>
       <c r="B69" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C69" s="51">
         <v>0</v>
@@ -11743,7 +11796,7 @@
         <v>32</v>
       </c>
       <c r="B70" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C70" s="51">
         <v>0</v>
@@ -11781,7 +11834,7 @@
         <v>33</v>
       </c>
       <c r="B71" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C71" s="51">
         <v>0</v>
@@ -11819,7 +11872,7 @@
         <v>34</v>
       </c>
       <c r="B72" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C72" s="51">
         <v>0</v>
@@ -11857,7 +11910,7 @@
         <v>35</v>
       </c>
       <c r="B73" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C73" s="51">
         <v>0</v>
@@ -11895,7 +11948,7 @@
         <v>36</v>
       </c>
       <c r="B74" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C74" s="51">
         <v>0</v>
@@ -11933,7 +11986,7 @@
         <v>37</v>
       </c>
       <c r="B75" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C75" s="51">
         <v>0</v>
@@ -11971,7 +12024,7 @@
         <v>38</v>
       </c>
       <c r="B76" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C76" s="51">
         <v>0</v>
@@ -12009,7 +12062,7 @@
         <v>39</v>
       </c>
       <c r="B77" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C77" s="51">
         <v>0</v>
@@ -12047,7 +12100,7 @@
         <v>40</v>
       </c>
       <c r="B78" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C78" s="51">
         <v>0</v>
@@ -12085,7 +12138,7 @@
         <v>41</v>
       </c>
       <c r="B79" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C79" s="51">
         <v>0</v>
@@ -12123,7 +12176,7 @@
         <v>42</v>
       </c>
       <c r="B80" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C80" s="51">
         <v>0</v>
@@ -12161,7 +12214,7 @@
         <v>43</v>
       </c>
       <c r="B81" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C81" s="51">
         <v>0</v>
@@ -12199,7 +12252,7 @@
         <v>44</v>
       </c>
       <c r="B82" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C82" s="51">
         <v>0</v>
@@ -12237,7 +12290,7 @@
         <v>45</v>
       </c>
       <c r="B83" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C83" s="51">
         <v>0</v>
@@ -12275,7 +12328,7 @@
         <v>46</v>
       </c>
       <c r="B84" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C84" s="51">
         <v>0</v>
@@ -12313,7 +12366,7 @@
         <v>47</v>
       </c>
       <c r="B85" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C85" s="51">
         <v>0</v>
@@ -12351,7 +12404,7 @@
         <v>48</v>
       </c>
       <c r="B86" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C86" s="51">
         <v>0</v>
@@ -12389,7 +12442,7 @@
         <v>49</v>
       </c>
       <c r="B87" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C87" s="51">
         <v>0</v>
@@ -12427,7 +12480,7 @@
         <v>50</v>
       </c>
       <c r="B88" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C88" s="51">
         <v>0</v>
@@ -12465,7 +12518,7 @@
         <v>51</v>
       </c>
       <c r="B89" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C89" s="51">
         <v>0</v>
@@ -12503,7 +12556,7 @@
         <v>52</v>
       </c>
       <c r="B90" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C90" s="51">
         <v>0</v>
@@ -12541,7 +12594,7 @@
         <v>53</v>
       </c>
       <c r="B91" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C91" s="51">
         <v>0</v>
@@ -12579,7 +12632,7 @@
         <v>54</v>
       </c>
       <c r="B92" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C92" s="51">
         <v>0</v>
@@ -12617,7 +12670,7 @@
         <v>55</v>
       </c>
       <c r="B93" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C93" s="51">
         <v>0</v>
@@ -12655,7 +12708,7 @@
         <v>56</v>
       </c>
       <c r="B94" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C94" s="51">
         <v>0</v>
@@ -12693,7 +12746,7 @@
         <v>57</v>
       </c>
       <c r="B95" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C95" s="51">
         <v>0</v>
@@ -12731,7 +12784,7 @@
         <v>58</v>
       </c>
       <c r="B96" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C96" s="51">
         <v>0</v>
@@ -12769,7 +12822,7 @@
         <v>59</v>
       </c>
       <c r="B97" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C97" s="51">
         <v>0</v>
@@ -12807,7 +12860,7 @@
         <v>60</v>
       </c>
       <c r="B98" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C98" s="51">
         <v>0</v>
@@ -12845,7 +12898,7 @@
         <v>61</v>
       </c>
       <c r="B99" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C99" s="51">
         <v>0.01</v>
@@ -12883,7 +12936,7 @@
         <v>62</v>
       </c>
       <c r="B100" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C100" s="51">
         <v>0.01</v>
@@ -12921,7 +12974,7 @@
         <v>63</v>
       </c>
       <c r="B101" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C101" s="51">
         <v>0.01</v>
@@ -12959,7 +13012,7 @@
         <v>64</v>
       </c>
       <c r="B102" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C102" s="51">
         <v>0.01</v>
@@ -12997,7 +13050,7 @@
         <v>65</v>
       </c>
       <c r="B103" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C103" s="51">
         <v>0.01</v>
@@ -13035,7 +13088,7 @@
         <v>66</v>
       </c>
       <c r="B104" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C104" s="51">
         <v>0.01</v>
@@ -13073,7 +13126,7 @@
         <v>67</v>
       </c>
       <c r="B105" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C105" s="51">
         <v>0.01</v>
@@ -13111,7 +13164,7 @@
         <v>68</v>
       </c>
       <c r="B106" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C106" s="51">
         <v>0.01</v>
@@ -13149,7 +13202,7 @@
         <v>69</v>
       </c>
       <c r="B107" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C107" s="51">
         <v>0.01</v>
@@ -13187,7 +13240,7 @@
         <v>70</v>
       </c>
       <c r="B108" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C108" s="51">
         <v>0.01</v>
@@ -13225,7 +13278,7 @@
         <v>71</v>
       </c>
       <c r="B109" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C109" s="51">
         <v>0.01</v>
@@ -13263,7 +13316,7 @@
         <v>72</v>
       </c>
       <c r="B110" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C110" s="51">
         <v>0.01</v>
@@ -13301,7 +13354,7 @@
         <v>73</v>
       </c>
       <c r="B111" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C111" s="51">
         <v>0.02</v>
@@ -13339,7 +13392,7 @@
         <v>74</v>
       </c>
       <c r="B112" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C112" s="51">
         <v>0.02</v>
@@ -13377,7 +13430,7 @@
         <v>75</v>
       </c>
       <c r="B113" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C113" s="51">
         <v>0.02</v>
@@ -13415,7 +13468,7 @@
         <v>76</v>
       </c>
       <c r="B114" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C114" s="51">
         <v>0.02</v>
@@ -13453,7 +13506,7 @@
         <v>77</v>
       </c>
       <c r="B115" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C115" s="51">
         <v>0.03</v>
@@ -13491,7 +13544,7 @@
         <v>78</v>
       </c>
       <c r="B116" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C116" s="51">
         <v>0.03</v>
@@ -13529,7 +13582,7 @@
         <v>79</v>
       </c>
       <c r="B117" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C117" s="51">
         <v>0.03</v>
@@ -13567,7 +13620,7 @@
         <v>80</v>
       </c>
       <c r="B118" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C118" s="51">
         <v>0.04</v>
@@ -13605,7 +13658,7 @@
         <v>81</v>
       </c>
       <c r="B119" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C119" s="51">
         <v>0.04</v>
@@ -13643,7 +13696,7 @@
         <v>82</v>
       </c>
       <c r="B120" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C120" s="51">
         <v>0.05</v>
@@ -13681,7 +13734,7 @@
         <v>83</v>
       </c>
       <c r="B121" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C121" s="51">
         <v>0.05</v>
@@ -13719,7 +13772,7 @@
         <v>84</v>
       </c>
       <c r="B122" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C122" s="51">
         <v>0.06</v>
@@ -13757,7 +13810,7 @@
         <v>85</v>
       </c>
       <c r="B123" s="51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C123" s="51">
         <v>7.0000000000000007E-2</v>
@@ -13898,7 +13951,7 @@
     </row>
     <row r="9" spans="1:5" ht="17.100000000000001" customHeight="1">
       <c r="A9" s="61" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B9" s="61"/>
       <c r="C9" s="62" t="s">
@@ -13909,7 +13962,7 @@
     </row>
     <row r="10" spans="1:5" ht="17.100000000000001" customHeight="1">
       <c r="A10" s="61" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B10" s="61"/>
       <c r="C10" s="62" t="s">
@@ -14001,7 +14054,7 @@
         <v>47</v>
       </c>
       <c r="D2" s="42" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E2" s="52">
         <v>0</v>
@@ -14013,7 +14066,7 @@
         <v>50</v>
       </c>
       <c r="H2" s="45" t="s">
-        <v>127</v>
+        <v>146</v>
       </c>
       <c r="I2" s="43">
         <v>50</v>
@@ -14037,7 +14090,7 @@
       </c>
       <c r="C3" s="4"/>
       <c r="D3" s="9" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E3" s="53">
         <v>1.2430000000000001</v>
@@ -14068,7 +14121,7 @@
       </c>
       <c r="C4" s="4"/>
       <c r="D4" s="9" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="E4" s="53">
         <v>1.6479999999999999</v>
@@ -14099,7 +14152,7 @@
       </c>
       <c r="C5" s="4"/>
       <c r="D5" s="9" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E5" s="53">
         <v>1.6479999999999999</v>
@@ -14280,7 +14333,7 @@
       </c>
       <c r="G11" s="4"/>
       <c r="H11" s="48" t="s">
-        <v>88</v>
+        <v>147</v>
       </c>
       <c r="I11" s="25">
         <v>70</v>
@@ -14512,7 +14565,7 @@
       </c>
       <c r="G19" s="4"/>
       <c r="H19" s="49" t="s">
-        <v>102</v>
+        <v>148</v>
       </c>
       <c r="I19" s="25">
         <v>90</v>
@@ -14574,7 +14627,7 @@
       </c>
       <c r="G21" s="4"/>
       <c r="H21" s="49" t="s">
-        <v>107</v>
+        <v>150</v>
       </c>
       <c r="I21" s="25">
         <v>100</v>
@@ -14592,13 +14645,13 @@
         <v>34</v>
       </c>
       <c r="B22" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="C22" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="D22" s="9" t="s">
         <v>109</v>
-      </c>
-      <c r="D22" s="9" t="s">
-        <v>110</v>
       </c>
       <c r="E22" s="53">
         <v>0</v>
@@ -14614,7 +14667,7 @@
       <c r="J22" s="4"/>
       <c r="K22" s="4"/>
       <c r="L22" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="M22" s="4"/>
       <c r="N22" s="44">
@@ -14626,11 +14679,11 @@
         <v>34</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C23" s="9"/>
       <c r="D23" s="9" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E23" s="53">
         <v>0</v>
@@ -14646,7 +14699,7 @@
       <c r="J23" s="4"/>
       <c r="K23" s="4"/>
       <c r="L23" s="9" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="M23" s="4"/>
       <c r="N23" s="44">
@@ -14655,20 +14708,20 @@
     </row>
     <row r="24" spans="1:14" ht="15.75" customHeight="1">
       <c r="A24" s="9" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B24" s="9"/>
       <c r="C24" s="9" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D24" s="9"/>
       <c r="E24" s="53"/>
       <c r="F24" s="9" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="G24" s="4"/>
       <c r="H24" s="49" t="s">
-        <v>107</v>
+        <v>149</v>
       </c>
       <c r="I24" s="25">
         <v>120</v>
@@ -14683,16 +14736,16 @@
     </row>
     <row r="25" spans="1:14" ht="30">
       <c r="A25" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="D25" s="25" t="s">
         <v>134</v>
-      </c>
-      <c r="B25" s="9" t="s">
-        <v>145</v>
-      </c>
-      <c r="C25" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="D25" s="25" t="s">
-        <v>136</v>
       </c>
       <c r="E25" s="53">
         <v>0</v>
@@ -14702,7 +14755,7 @@
       </c>
       <c r="G25" s="4"/>
       <c r="H25" s="49" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="I25" s="25">
         <v>130</v>
@@ -14719,14 +14772,14 @@
     </row>
     <row r="26" spans="1:14" ht="17.100000000000001" customHeight="1">
       <c r="A26" s="9" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C26" s="4"/>
       <c r="D26" s="25" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E26" s="53">
         <v>1</v>
@@ -14751,14 +14804,14 @@
     </row>
     <row r="27" spans="1:14" ht="17.100000000000001" customHeight="1">
       <c r="A27" s="9" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C27" s="4"/>
       <c r="D27" s="25" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="E27" s="53">
         <v>2</v>

</xml_diff>

<commit_message>
KCP-101 - numeric validation text
</commit_message>
<xml_diff>
--- a/resources/kcp-models-master.xlsx
+++ b/resources/kcp-models-master.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\kcp2\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{217B294A-7196-43DD-95BD-C45F3F20F84B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFD51361-C56E-4901-AD12-A9B8DCCF674D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -502,9 +502,6 @@
     <t>Age at surgery</t>
   </si>
   <si>
-    <t>{:dps 0, :max 85, :min 25, :type :numeric}</t>
-  </si>
-  <si>
     <t>:Male</t>
   </si>
   <si>
@@ -575,9 +572,6 @@
   </si>
   <si>
     <t>Charlson comorbidity score</t>
-  </si>
-  <si>
-    <t>{:dps 0, :max 31, :min 2, :type :numeric}</t>
   </si>
   <si>
     <t>:smoking-history</t>
@@ -705,6 +699,12 @@
   </si>
   <si>
     <t>[:p "Age when the kidney cancer surgery was performed. Older patients are more at risk of other long-term health conditions and are relatively less likely to die from kidney cancer. An age between 25 and 85 may be entered here."]</t>
+  </si>
+  <si>
+    <t>{:dps 0, :max 31, :min 2, :type :numeric :validation "Score must be between 2 and 31"}</t>
+  </si>
+  <si>
+    <t>{:dps 0, :max 85, :min 25, :type :numeric :validation "Age must be between 25 and 85 years"}</t>
   </si>
 </sst>
 </file>
@@ -2314,13 +2314,13 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
+        <v>136</v>
+      </c>
+      <c r="B1" t="s">
+        <v>137</v>
+      </c>
+      <c r="C1" t="s">
         <v>138</v>
-      </c>
-      <c r="B1" t="s">
-        <v>139</v>
-      </c>
-      <c r="C1" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -2342,7 +2342,7 @@
         <v>0.42</v>
       </c>
       <c r="C3" s="54" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -4282,13 +4282,13 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
+        <v>136</v>
+      </c>
+      <c r="B1" t="s">
+        <v>137</v>
+      </c>
+      <c r="C1" t="s">
         <v>138</v>
-      </c>
-      <c r="B1" t="s">
-        <v>139</v>
-      </c>
-      <c r="C1" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -6415,7 +6415,7 @@
     </row>
     <row r="3" spans="1:5" ht="17.100000000000001" customHeight="1">
       <c r="A3" s="23" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B3" s="21" t="s">
         <v>19</v>
@@ -9072,11 +9072,11 @@
       <c r="D25" s="9"/>
       <c r="E25" s="53"/>
       <c r="F25" s="9" t="s">
-        <v>106</v>
+        <v>150</v>
       </c>
       <c r="G25" s="4"/>
       <c r="H25" s="49" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="I25" s="25">
         <v>100</v>
@@ -9094,13 +9094,13 @@
         <v>34</v>
       </c>
       <c r="B26" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="C26" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="D26" s="9" t="s">
         <v>108</v>
-      </c>
-      <c r="D26" s="9" t="s">
-        <v>109</v>
       </c>
       <c r="E26" s="53">
         <v>0</v>
@@ -9116,7 +9116,7 @@
       <c r="J26" s="4"/>
       <c r="K26" s="4"/>
       <c r="L26" s="9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="M26" s="4"/>
       <c r="N26" s="44">
@@ -9128,11 +9128,11 @@
         <v>34</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C27" s="9"/>
       <c r="D27" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E27" s="53">
         <v>0</v>
@@ -9148,7 +9148,7 @@
       <c r="J27" s="4"/>
       <c r="K27" s="4"/>
       <c r="L27" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="M27" s="4"/>
       <c r="N27" s="44">
@@ -9171,40 +9171,40 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="50" t="s">
+        <v>111</v>
+      </c>
+      <c r="B1" s="50" t="s">
+        <v>107</v>
+      </c>
+      <c r="C1" s="50" t="s">
         <v>112</v>
       </c>
-      <c r="B1" s="50" t="s">
-        <v>108</v>
-      </c>
-      <c r="C1" s="50" t="s">
+      <c r="D1" s="50" t="s">
         <v>113</v>
       </c>
-      <c r="D1" s="50" t="s">
+      <c r="E1" s="50" t="s">
         <v>114</v>
       </c>
-      <c r="E1" s="50" t="s">
+      <c r="F1" s="50" t="s">
         <v>115</v>
       </c>
-      <c r="F1" s="50" t="s">
+      <c r="G1" s="50" t="s">
         <v>116</v>
       </c>
-      <c r="G1" s="50" t="s">
+      <c r="H1" s="50" t="s">
         <v>117</v>
       </c>
-      <c r="H1" s="50" t="s">
+      <c r="I1" s="50" t="s">
         <v>118</v>
       </c>
-      <c r="I1" s="50" t="s">
+      <c r="J1" s="50" t="s">
         <v>119</v>
       </c>
-      <c r="J1" s="50" t="s">
+      <c r="K1" s="50" t="s">
         <v>120</v>
       </c>
-      <c r="K1" s="50" t="s">
+      <c r="L1" s="50" t="s">
         <v>121</v>
-      </c>
-      <c r="L1" s="50" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="2" spans="1:12">
@@ -9212,7 +9212,7 @@
         <v>25</v>
       </c>
       <c r="B2" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C2" s="51">
         <v>0</v>
@@ -9250,7 +9250,7 @@
         <v>26</v>
       </c>
       <c r="B3" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C3" s="51">
         <v>0</v>
@@ -9288,7 +9288,7 @@
         <v>27</v>
       </c>
       <c r="B4" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C4" s="51">
         <v>0</v>
@@ -9326,7 +9326,7 @@
         <v>28</v>
       </c>
       <c r="B5" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C5" s="51">
         <v>0</v>
@@ -9364,7 +9364,7 @@
         <v>29</v>
       </c>
       <c r="B6" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C6" s="51">
         <v>0</v>
@@ -9402,7 +9402,7 @@
         <v>30</v>
       </c>
       <c r="B7" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C7" s="51">
         <v>0</v>
@@ -9440,7 +9440,7 @@
         <v>31</v>
       </c>
       <c r="B8" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C8" s="51">
         <v>0</v>
@@ -9478,7 +9478,7 @@
         <v>32</v>
       </c>
       <c r="B9" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C9" s="51">
         <v>0</v>
@@ -9516,7 +9516,7 @@
         <v>33</v>
       </c>
       <c r="B10" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C10" s="51">
         <v>0</v>
@@ -9554,7 +9554,7 @@
         <v>34</v>
       </c>
       <c r="B11" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C11" s="51">
         <v>0</v>
@@ -9592,7 +9592,7 @@
         <v>35</v>
       </c>
       <c r="B12" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C12" s="51">
         <v>0</v>
@@ -9630,7 +9630,7 @@
         <v>36</v>
       </c>
       <c r="B13" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C13" s="51">
         <v>0</v>
@@ -9668,7 +9668,7 @@
         <v>37</v>
       </c>
       <c r="B14" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C14" s="51">
         <v>0</v>
@@ -9706,7 +9706,7 @@
         <v>38</v>
       </c>
       <c r="B15" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C15" s="51">
         <v>0</v>
@@ -9744,7 +9744,7 @@
         <v>39</v>
       </c>
       <c r="B16" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C16" s="51">
         <v>0</v>
@@ -9782,7 +9782,7 @@
         <v>40</v>
       </c>
       <c r="B17" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C17" s="51">
         <v>0</v>
@@ -9820,7 +9820,7 @@
         <v>41</v>
       </c>
       <c r="B18" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C18" s="51">
         <v>0</v>
@@ -9858,7 +9858,7 @@
         <v>42</v>
       </c>
       <c r="B19" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C19" s="51">
         <v>0</v>
@@ -9896,7 +9896,7 @@
         <v>43</v>
       </c>
       <c r="B20" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C20" s="51">
         <v>0</v>
@@ -9934,7 +9934,7 @@
         <v>44</v>
       </c>
       <c r="B21" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C21" s="51">
         <v>0</v>
@@ -9972,7 +9972,7 @@
         <v>45</v>
       </c>
       <c r="B22" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C22" s="51">
         <v>0</v>
@@ -10010,7 +10010,7 @@
         <v>46</v>
       </c>
       <c r="B23" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C23" s="51">
         <v>0</v>
@@ -10048,7 +10048,7 @@
         <v>47</v>
       </c>
       <c r="B24" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C24" s="51">
         <v>0</v>
@@ -10086,7 +10086,7 @@
         <v>48</v>
       </c>
       <c r="B25" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C25" s="51">
         <v>0</v>
@@ -10124,7 +10124,7 @@
         <v>49</v>
       </c>
       <c r="B26" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C26" s="51">
         <v>0</v>
@@ -10162,7 +10162,7 @@
         <v>50</v>
       </c>
       <c r="B27" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C27" s="51">
         <v>0</v>
@@ -10200,7 +10200,7 @@
         <v>51</v>
       </c>
       <c r="B28" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C28" s="51">
         <v>0</v>
@@ -10238,7 +10238,7 @@
         <v>52</v>
       </c>
       <c r="B29" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C29" s="51">
         <v>0</v>
@@ -10276,7 +10276,7 @@
         <v>53</v>
       </c>
       <c r="B30" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C30" s="51">
         <v>0</v>
@@ -10314,7 +10314,7 @@
         <v>54</v>
       </c>
       <c r="B31" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C31" s="51">
         <v>0</v>
@@ -10352,7 +10352,7 @@
         <v>55</v>
       </c>
       <c r="B32" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C32" s="51">
         <v>0</v>
@@ -10390,7 +10390,7 @@
         <v>56</v>
       </c>
       <c r="B33" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C33" s="51">
         <v>0.01</v>
@@ -10428,7 +10428,7 @@
         <v>57</v>
       </c>
       <c r="B34" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C34" s="51">
         <v>0.01</v>
@@ -10466,7 +10466,7 @@
         <v>58</v>
       </c>
       <c r="B35" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C35" s="51">
         <v>0.01</v>
@@ -10504,7 +10504,7 @@
         <v>59</v>
       </c>
       <c r="B36" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C36" s="51">
         <v>0.01</v>
@@ -10542,7 +10542,7 @@
         <v>60</v>
       </c>
       <c r="B37" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C37" s="51">
         <v>0.01</v>
@@ -10580,7 +10580,7 @@
         <v>61</v>
       </c>
       <c r="B38" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C38" s="51">
         <v>0.01</v>
@@ -10618,7 +10618,7 @@
         <v>62</v>
       </c>
       <c r="B39" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C39" s="51">
         <v>0.01</v>
@@ -10656,7 +10656,7 @@
         <v>63</v>
       </c>
       <c r="B40" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C40" s="51">
         <v>0.01</v>
@@ -10694,7 +10694,7 @@
         <v>64</v>
       </c>
       <c r="B41" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C41" s="51">
         <v>0.01</v>
@@ -10732,7 +10732,7 @@
         <v>65</v>
       </c>
       <c r="B42" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C42" s="51">
         <v>0.01</v>
@@ -10770,7 +10770,7 @@
         <v>66</v>
       </c>
       <c r="B43" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C43" s="51">
         <v>0.01</v>
@@ -10808,7 +10808,7 @@
         <v>67</v>
       </c>
       <c r="B44" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C44" s="51">
         <v>0.01</v>
@@ -10846,7 +10846,7 @@
         <v>68</v>
       </c>
       <c r="B45" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C45" s="51">
         <v>0.02</v>
@@ -10884,7 +10884,7 @@
         <v>69</v>
       </c>
       <c r="B46" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C46" s="51">
         <v>0.02</v>
@@ -10922,7 +10922,7 @@
         <v>70</v>
       </c>
       <c r="B47" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C47" s="51">
         <v>0.02</v>
@@ -10960,7 +10960,7 @@
         <v>71</v>
       </c>
       <c r="B48" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C48" s="51">
         <v>0.02</v>
@@ -10998,7 +10998,7 @@
         <v>72</v>
       </c>
       <c r="B49" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C49" s="51">
         <v>0.02</v>
@@ -11036,7 +11036,7 @@
         <v>73</v>
       </c>
       <c r="B50" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C50" s="51">
         <v>0.02</v>
@@ -11074,7 +11074,7 @@
         <v>74</v>
       </c>
       <c r="B51" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C51" s="51">
         <v>0.03</v>
@@ -11112,7 +11112,7 @@
         <v>75</v>
       </c>
       <c r="B52" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C52" s="51">
         <v>0.03</v>
@@ -11150,7 +11150,7 @@
         <v>76</v>
       </c>
       <c r="B53" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C53" s="51">
         <v>0.03</v>
@@ -11188,7 +11188,7 @@
         <v>77</v>
       </c>
       <c r="B54" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C54" s="51">
         <v>0.04</v>
@@ -11226,7 +11226,7 @@
         <v>78</v>
       </c>
       <c r="B55" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C55" s="51">
         <v>0.04</v>
@@ -11264,7 +11264,7 @@
         <v>79</v>
       </c>
       <c r="B56" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C56" s="51">
         <v>0.05</v>
@@ -11302,7 +11302,7 @@
         <v>80</v>
       </c>
       <c r="B57" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C57" s="51">
         <v>0.05</v>
@@ -11340,7 +11340,7 @@
         <v>81</v>
       </c>
       <c r="B58" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C58" s="51">
         <v>0.06</v>
@@ -11378,7 +11378,7 @@
         <v>82</v>
       </c>
       <c r="B59" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C59" s="51">
         <v>7.0000000000000007E-2</v>
@@ -11416,7 +11416,7 @@
         <v>83</v>
       </c>
       <c r="B60" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C60" s="51">
         <v>7.0000000000000007E-2</v>
@@ -11454,7 +11454,7 @@
         <v>84</v>
       </c>
       <c r="B61" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C61" s="51">
         <v>0.08</v>
@@ -11492,7 +11492,7 @@
         <v>85</v>
       </c>
       <c r="B62" s="51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C62" s="51">
         <v>0.09</v>
@@ -11530,7 +11530,7 @@
         <v>25</v>
       </c>
       <c r="B63" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C63" s="51">
         <v>0</v>
@@ -11568,7 +11568,7 @@
         <v>26</v>
       </c>
       <c r="B64" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C64" s="51">
         <v>0</v>
@@ -11606,7 +11606,7 @@
         <v>27</v>
       </c>
       <c r="B65" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C65" s="51">
         <v>0</v>
@@ -11644,7 +11644,7 @@
         <v>28</v>
       </c>
       <c r="B66" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C66" s="51">
         <v>0</v>
@@ -11682,7 +11682,7 @@
         <v>29</v>
       </c>
       <c r="B67" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C67" s="51">
         <v>0</v>
@@ -11720,7 +11720,7 @@
         <v>30</v>
       </c>
       <c r="B68" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C68" s="51">
         <v>0</v>
@@ -11758,7 +11758,7 @@
         <v>31</v>
       </c>
       <c r="B69" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C69" s="51">
         <v>0</v>
@@ -11796,7 +11796,7 @@
         <v>32</v>
       </c>
       <c r="B70" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C70" s="51">
         <v>0</v>
@@ -11834,7 +11834,7 @@
         <v>33</v>
       </c>
       <c r="B71" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C71" s="51">
         <v>0</v>
@@ -11872,7 +11872,7 @@
         <v>34</v>
       </c>
       <c r="B72" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C72" s="51">
         <v>0</v>
@@ -11910,7 +11910,7 @@
         <v>35</v>
       </c>
       <c r="B73" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C73" s="51">
         <v>0</v>
@@ -11948,7 +11948,7 @@
         <v>36</v>
       </c>
       <c r="B74" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C74" s="51">
         <v>0</v>
@@ -11986,7 +11986,7 @@
         <v>37</v>
       </c>
       <c r="B75" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C75" s="51">
         <v>0</v>
@@ -12024,7 +12024,7 @@
         <v>38</v>
       </c>
       <c r="B76" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C76" s="51">
         <v>0</v>
@@ -12062,7 +12062,7 @@
         <v>39</v>
       </c>
       <c r="B77" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C77" s="51">
         <v>0</v>
@@ -12100,7 +12100,7 @@
         <v>40</v>
       </c>
       <c r="B78" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C78" s="51">
         <v>0</v>
@@ -12138,7 +12138,7 @@
         <v>41</v>
       </c>
       <c r="B79" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C79" s="51">
         <v>0</v>
@@ -12176,7 +12176,7 @@
         <v>42</v>
       </c>
       <c r="B80" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C80" s="51">
         <v>0</v>
@@ -12214,7 +12214,7 @@
         <v>43</v>
       </c>
       <c r="B81" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C81" s="51">
         <v>0</v>
@@ -12252,7 +12252,7 @@
         <v>44</v>
       </c>
       <c r="B82" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C82" s="51">
         <v>0</v>
@@ -12290,7 +12290,7 @@
         <v>45</v>
       </c>
       <c r="B83" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C83" s="51">
         <v>0</v>
@@ -12328,7 +12328,7 @@
         <v>46</v>
       </c>
       <c r="B84" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C84" s="51">
         <v>0</v>
@@ -12366,7 +12366,7 @@
         <v>47</v>
       </c>
       <c r="B85" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C85" s="51">
         <v>0</v>
@@ -12404,7 +12404,7 @@
         <v>48</v>
       </c>
       <c r="B86" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C86" s="51">
         <v>0</v>
@@ -12442,7 +12442,7 @@
         <v>49</v>
       </c>
       <c r="B87" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C87" s="51">
         <v>0</v>
@@ -12480,7 +12480,7 @@
         <v>50</v>
       </c>
       <c r="B88" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C88" s="51">
         <v>0</v>
@@ -12518,7 +12518,7 @@
         <v>51</v>
       </c>
       <c r="B89" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C89" s="51">
         <v>0</v>
@@ -12556,7 +12556,7 @@
         <v>52</v>
       </c>
       <c r="B90" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C90" s="51">
         <v>0</v>
@@ -12594,7 +12594,7 @@
         <v>53</v>
       </c>
       <c r="B91" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C91" s="51">
         <v>0</v>
@@ -12632,7 +12632,7 @@
         <v>54</v>
       </c>
       <c r="B92" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C92" s="51">
         <v>0</v>
@@ -12670,7 +12670,7 @@
         <v>55</v>
       </c>
       <c r="B93" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C93" s="51">
         <v>0</v>
@@ -12708,7 +12708,7 @@
         <v>56</v>
       </c>
       <c r="B94" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C94" s="51">
         <v>0</v>
@@ -12746,7 +12746,7 @@
         <v>57</v>
       </c>
       <c r="B95" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C95" s="51">
         <v>0</v>
@@ -12784,7 +12784,7 @@
         <v>58</v>
       </c>
       <c r="B96" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C96" s="51">
         <v>0</v>
@@ -12822,7 +12822,7 @@
         <v>59</v>
       </c>
       <c r="B97" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C97" s="51">
         <v>0</v>
@@ -12860,7 +12860,7 @@
         <v>60</v>
       </c>
       <c r="B98" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C98" s="51">
         <v>0</v>
@@ -12898,7 +12898,7 @@
         <v>61</v>
       </c>
       <c r="B99" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C99" s="51">
         <v>0.01</v>
@@ -12936,7 +12936,7 @@
         <v>62</v>
       </c>
       <c r="B100" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C100" s="51">
         <v>0.01</v>
@@ -12974,7 +12974,7 @@
         <v>63</v>
       </c>
       <c r="B101" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C101" s="51">
         <v>0.01</v>
@@ -13012,7 +13012,7 @@
         <v>64</v>
       </c>
       <c r="B102" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C102" s="51">
         <v>0.01</v>
@@ -13050,7 +13050,7 @@
         <v>65</v>
       </c>
       <c r="B103" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C103" s="51">
         <v>0.01</v>
@@ -13088,7 +13088,7 @@
         <v>66</v>
       </c>
       <c r="B104" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C104" s="51">
         <v>0.01</v>
@@ -13126,7 +13126,7 @@
         <v>67</v>
       </c>
       <c r="B105" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C105" s="51">
         <v>0.01</v>
@@ -13164,7 +13164,7 @@
         <v>68</v>
       </c>
       <c r="B106" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C106" s="51">
         <v>0.01</v>
@@ -13202,7 +13202,7 @@
         <v>69</v>
       </c>
       <c r="B107" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C107" s="51">
         <v>0.01</v>
@@ -13240,7 +13240,7 @@
         <v>70</v>
       </c>
       <c r="B108" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C108" s="51">
         <v>0.01</v>
@@ -13278,7 +13278,7 @@
         <v>71</v>
       </c>
       <c r="B109" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C109" s="51">
         <v>0.01</v>
@@ -13316,7 +13316,7 @@
         <v>72</v>
       </c>
       <c r="B110" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C110" s="51">
         <v>0.01</v>
@@ -13354,7 +13354,7 @@
         <v>73</v>
       </c>
       <c r="B111" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C111" s="51">
         <v>0.02</v>
@@ -13392,7 +13392,7 @@
         <v>74</v>
       </c>
       <c r="B112" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C112" s="51">
         <v>0.02</v>
@@ -13430,7 +13430,7 @@
         <v>75</v>
       </c>
       <c r="B113" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C113" s="51">
         <v>0.02</v>
@@ -13468,7 +13468,7 @@
         <v>76</v>
       </c>
       <c r="B114" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C114" s="51">
         <v>0.02</v>
@@ -13506,7 +13506,7 @@
         <v>77</v>
       </c>
       <c r="B115" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C115" s="51">
         <v>0.03</v>
@@ -13544,7 +13544,7 @@
         <v>78</v>
       </c>
       <c r="B116" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C116" s="51">
         <v>0.03</v>
@@ -13582,7 +13582,7 @@
         <v>79</v>
       </c>
       <c r="B117" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C117" s="51">
         <v>0.03</v>
@@ -13620,7 +13620,7 @@
         <v>80</v>
       </c>
       <c r="B118" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C118" s="51">
         <v>0.04</v>
@@ -13658,7 +13658,7 @@
         <v>81</v>
       </c>
       <c r="B119" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C119" s="51">
         <v>0.04</v>
@@ -13696,7 +13696,7 @@
         <v>82</v>
       </c>
       <c r="B120" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C120" s="51">
         <v>0.05</v>
@@ -13734,7 +13734,7 @@
         <v>83</v>
       </c>
       <c r="B121" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C121" s="51">
         <v>0.05</v>
@@ -13772,7 +13772,7 @@
         <v>84</v>
       </c>
       <c r="B122" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C122" s="51">
         <v>0.06</v>
@@ -13810,7 +13810,7 @@
         <v>85</v>
       </c>
       <c r="B123" s="51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C123" s="51">
         <v>7.0000000000000007E-2</v>
@@ -13951,7 +13951,7 @@
     </row>
     <row r="9" spans="1:5" ht="17.100000000000001" customHeight="1">
       <c r="A9" s="61" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B9" s="61"/>
       <c r="C9" s="62" t="s">
@@ -13962,7 +13962,7 @@
     </row>
     <row r="10" spans="1:5" ht="17.100000000000001" customHeight="1">
       <c r="A10" s="61" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B10" s="61"/>
       <c r="C10" s="62" t="s">
@@ -14054,7 +14054,7 @@
         <v>47</v>
       </c>
       <c r="D2" s="42" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E2" s="52">
         <v>0</v>
@@ -14066,7 +14066,7 @@
         <v>50</v>
       </c>
       <c r="H2" s="45" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="I2" s="43">
         <v>50</v>
@@ -14090,7 +14090,7 @@
       </c>
       <c r="C3" s="4"/>
       <c r="D3" s="9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E3" s="53">
         <v>1.2430000000000001</v>
@@ -14121,7 +14121,7 @@
       </c>
       <c r="C4" s="4"/>
       <c r="D4" s="9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E4" s="53">
         <v>1.6479999999999999</v>
@@ -14152,7 +14152,7 @@
       </c>
       <c r="C5" s="4"/>
       <c r="D5" s="9" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E5" s="53">
         <v>1.6479999999999999</v>
@@ -14333,7 +14333,7 @@
       </c>
       <c r="G11" s="4"/>
       <c r="H11" s="48" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="I11" s="25">
         <v>70</v>
@@ -14565,7 +14565,7 @@
       </c>
       <c r="G19" s="4"/>
       <c r="H19" s="49" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I19" s="25">
         <v>90</v>
@@ -14623,11 +14623,11 @@
       <c r="D21" s="9"/>
       <c r="E21" s="53"/>
       <c r="F21" s="9" t="s">
-        <v>106</v>
+        <v>150</v>
       </c>
       <c r="G21" s="4"/>
       <c r="H21" s="49" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="I21" s="25">
         <v>100</v>
@@ -14645,13 +14645,13 @@
         <v>34</v>
       </c>
       <c r="B22" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="C22" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="D22" s="9" t="s">
         <v>108</v>
-      </c>
-      <c r="D22" s="9" t="s">
-        <v>109</v>
       </c>
       <c r="E22" s="53">
         <v>0</v>
@@ -14667,7 +14667,7 @@
       <c r="J22" s="4"/>
       <c r="K22" s="4"/>
       <c r="L22" s="9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="M22" s="4"/>
       <c r="N22" s="44">
@@ -14679,11 +14679,11 @@
         <v>34</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C23" s="9"/>
       <c r="D23" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E23" s="53">
         <v>0</v>
@@ -14699,7 +14699,7 @@
       <c r="J23" s="4"/>
       <c r="K23" s="4"/>
       <c r="L23" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="M23" s="4"/>
       <c r="N23" s="44">
@@ -14708,20 +14708,20 @@
     </row>
     <row r="24" spans="1:14" ht="15.75" customHeight="1">
       <c r="A24" s="9" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B24" s="9"/>
       <c r="C24" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D24" s="9"/>
       <c r="E24" s="53"/>
       <c r="F24" s="9" t="s">
-        <v>131</v>
+        <v>149</v>
       </c>
       <c r="G24" s="4"/>
       <c r="H24" s="49" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="I24" s="25">
         <v>120</v>
@@ -14736,16 +14736,16 @@
     </row>
     <row r="25" spans="1:14" ht="30">
       <c r="A25" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="D25" s="25" t="s">
         <v>132</v>
-      </c>
-      <c r="B25" s="9" t="s">
-        <v>143</v>
-      </c>
-      <c r="C25" s="9" t="s">
-        <v>133</v>
-      </c>
-      <c r="D25" s="25" t="s">
-        <v>134</v>
       </c>
       <c r="E25" s="53">
         <v>0</v>
@@ -14755,7 +14755,7 @@
       </c>
       <c r="G25" s="4"/>
       <c r="H25" s="49" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I25" s="25">
         <v>130</v>
@@ -14772,14 +14772,14 @@
     </row>
     <row r="26" spans="1:14" ht="17.100000000000001" customHeight="1">
       <c r="A26" s="9" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C26" s="4"/>
       <c r="D26" s="25" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E26" s="53">
         <v>1</v>
@@ -14804,14 +14804,14 @@
     </row>
     <row r="27" spans="1:14" ht="17.100000000000001" customHeight="1">
       <c r="A27" s="9" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C27" s="4"/>
       <c r="D27" s="25" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="E27" s="53">
         <v>2</v>

</xml_diff>

<commit_message>
KCP-101 - add calc workflow
</commit_message>
<xml_diff>
--- a/resources/kcp-models-master.xlsx
+++ b/resources/kcp-models-master.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\kcp2\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFD51361-C56E-4901-AD12-A9B8DCCF674D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14699D6F-B27B-4E84-AEE9-27FAE52DD042}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -701,10 +701,10 @@
     <t>[:p "Age when the kidney cancer surgery was performed. Older patients are more at risk of other long-term health conditions and are relatively less likely to die from kidney cancer. An age between 25 and 85 may be entered here."]</t>
   </si>
   <si>
-    <t>{:dps 0, :max 31, :min 2, :type :numeric :validation "Score must be between 2 and 31"}</t>
-  </si>
-  <si>
     <t>{:dps 0, :max 85, :min 25, :type :numeric :validation "Age must be between 25 and 85 years"}</t>
+  </si>
+  <si>
+    <t>{:dps 0, :max 31, :min 2, :type :numeric :validation "Score must be between 2 and 31"  :calc-workflow :charlson}</t>
   </si>
 </sst>
 </file>
@@ -9072,7 +9072,7 @@
       <c r="D25" s="9"/>
       <c r="E25" s="53"/>
       <c r="F25" s="9" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G25" s="4"/>
       <c r="H25" s="49" t="s">
@@ -14623,7 +14623,7 @@
       <c r="D21" s="9"/>
       <c r="E21" s="53"/>
       <c r="F21" s="9" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G21" s="4"/>
       <c r="H21" s="49" t="s">
@@ -14717,7 +14717,7 @@
       <c r="D24" s="9"/>
       <c r="E24" s="53"/>
       <c r="F24" s="9" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G24" s="4"/>
       <c r="H24" s="49" t="s">

</xml_diff>

<commit_message>
KCP-101 - correct tobacco label
</commit_message>
<xml_diff>
--- a/resources/kcp-models-master.xlsx
+++ b/resources/kcp-models-master.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\kcp2\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\kcp\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14699D6F-B27B-4E84-AEE9-27FAE52DD042}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B56A9581-4766-4D3C-9198-22122D9BB762}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="38700" windowHeight="15285" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -609,9 +609,6 @@
     <t>Former tobacco use</t>
   </si>
   <si>
-    <t xml:space="preserve">Never Used Tobacco </t>
-  </si>
-  <si>
     <t>Index</t>
   </si>
   <si>
@@ -706,6 +703,9 @@
   <si>
     <t>{:dps 0, :max 31, :min 2, :type :numeric :validation "Score must be between 2 and 31"  :calc-workflow :charlson}</t>
   </si>
+  <si>
+    <t>Never used tobacco</t>
+  </si>
 </sst>
 </file>
 
@@ -714,7 +714,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="12"/>
       <color indexed="8"/>
@@ -785,6 +785,12 @@
       <sz val="11"/>
       <color indexed="8"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1F2328"/>
+      <name val="Segoe UI"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -956,7 +962,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1058,6 +1064,7 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2201,12 +2208,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="44" style="1" customWidth="1"/>
     <col min="2" max="2" width="26" style="1" customWidth="1"/>
-    <col min="3" max="6" width="8.6328125" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.6328125" style="1"/>
+    <col min="3" max="6" width="8.6640625" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.6640625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.100000000000001" customHeight="1">
@@ -2314,13 +2321,13 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1" t="s">
         <v>136</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>137</v>
-      </c>
-      <c r="C1" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -2342,7 +2349,7 @@
         <v>0.42</v>
       </c>
       <c r="C3" s="54" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -4282,13 +4289,13 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1" t="s">
         <v>136</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>137</v>
-      </c>
-      <c r="C1" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -6246,19 +6253,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F10"/>
-  <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="8.44140625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="8.453125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="14.453125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="28.36328125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="24.81640625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="33.6328125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="22.453125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="8.453125" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.453125" style="1"/>
+    <col min="1" max="1" width="8.44140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="14.44140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="28.33203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="24.77734375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="33.6640625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="22.44140625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="8.44140625" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.44140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.45" customHeight="1">
+    <row r="1" spans="1:6" ht="15.4" customHeight="1">
       <c r="A1" s="10" t="s">
         <v>6</v>
       </c>
@@ -6278,7 +6285,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="17.399999999999999" customHeight="1">
+    <row r="2" spans="1:6" ht="17.45" customHeight="1">
       <c r="A2" s="10" t="s">
         <v>12</v>
       </c>
@@ -6377,14 +6384,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="8.44140625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="7.453125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="19.36328125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="15.36328125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="14.453125" style="1" customWidth="1"/>
-    <col min="5" max="6" width="8.453125" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.453125" style="1"/>
+    <col min="1" max="1" width="7.44140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="19.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="15.33203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="14.44140625" style="1" customWidth="1"/>
+    <col min="5" max="6" width="8.44140625" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.44140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.100000000000001" customHeight="1">
@@ -6415,7 +6422,7 @@
     </row>
     <row r="3" spans="1:5" ht="17.100000000000001" customHeight="1">
       <c r="A3" s="23" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B3" s="21" t="s">
         <v>19</v>
@@ -6487,13 +6494,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E203"/>
-  <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="8.44140625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="14.90625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="7.453125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="13.1796875" style="1" customWidth="1"/>
-    <col min="4" max="6" width="8.453125" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.453125" style="1"/>
+    <col min="1" max="1" width="14.88671875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="7.44140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="13.21875" style="1" customWidth="1"/>
+    <col min="4" max="6" width="8.44140625" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.44140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.100000000000001" customHeight="1">
@@ -8182,12 +8189,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="8.44140625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16" style="1" customWidth="1"/>
-    <col min="2" max="2" width="13.36328125" style="1" customWidth="1"/>
-    <col min="3" max="6" width="8.453125" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.453125" style="1"/>
+    <col min="2" max="2" width="13.33203125" style="1" customWidth="1"/>
+    <col min="3" max="6" width="8.44140625" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.44140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.100000000000001" customHeight="1">
@@ -8306,21 +8313,21 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:N27"/>
-  <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="8.44140625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="16.6328125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.36328125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="10.33203125" style="1" customWidth="1"/>
     <col min="3" max="3" width="31" style="1" customWidth="1"/>
     <col min="4" max="4" width="43" style="1" customWidth="1"/>
-    <col min="5" max="5" width="15.36328125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="15.08984375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="15.33203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="15.109375" style="1" customWidth="1"/>
     <col min="7" max="7" width="81" style="1" customWidth="1"/>
-    <col min="8" max="8" width="116.36328125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="5.1796875" style="1" customWidth="1"/>
-    <col min="10" max="12" width="14.1796875" style="1" customWidth="1"/>
-    <col min="13" max="13" width="40.36328125" style="1" customWidth="1"/>
-    <col min="14" max="15" width="8.453125" style="1" customWidth="1"/>
-    <col min="16" max="16384" width="8.453125" style="1"/>
+    <col min="8" max="8" width="116.33203125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="5.21875" style="1" customWidth="1"/>
+    <col min="10" max="12" width="14.21875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="40.33203125" style="1" customWidth="1"/>
+    <col min="14" max="15" width="8.44140625" style="1" customWidth="1"/>
+    <col min="16" max="16384" width="8.44140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="17.100000000000001" customHeight="1">
@@ -8367,7 +8374,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="156.9" customHeight="1">
+    <row r="2" spans="1:14" ht="156.94999999999999" customHeight="1">
       <c r="A2" s="42" t="s">
         <v>30</v>
       </c>
@@ -8993,7 +9000,7 @@
       <c r="M22" s="4"/>
       <c r="N22" s="16"/>
     </row>
-    <row r="23" spans="1:14" ht="45.45" customHeight="1">
+    <row r="23" spans="1:14" ht="45.4" customHeight="1">
       <c r="A23" s="9" t="s">
         <v>32</v>
       </c>
@@ -9072,11 +9079,11 @@
       <c r="D25" s="9"/>
       <c r="E25" s="53"/>
       <c r="F25" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G25" s="4"/>
       <c r="H25" s="49" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="I25" s="25">
         <v>100</v>
@@ -9169,7 +9176,7 @@
   <dimension ref="A1:L123"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:12" ht="15.75">
       <c r="A1" s="50" t="s">
         <v>111</v>
       </c>
@@ -13851,12 +13858,12 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD640821-0FB9-4D59-BBAC-F550C45F339E}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="8.44140625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16" style="1" customWidth="1"/>
-    <col min="2" max="2" width="13.36328125" style="1" customWidth="1"/>
-    <col min="3" max="6" width="8.453125" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.453125" style="1"/>
+    <col min="2" max="2" width="13.33203125" style="1" customWidth="1"/>
+    <col min="3" max="6" width="8.44140625" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.44140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.100000000000001" customHeight="1">
@@ -13983,20 +13990,20 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{261E92C2-54DD-4827-851F-385906BB591F}">
   <dimension ref="A1:N27"/>
-  <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.44140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="16.6328125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.36328125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="10.33203125" style="1" customWidth="1"/>
     <col min="3" max="3" width="31" style="1" customWidth="1"/>
     <col min="4" max="4" width="43" style="1" customWidth="1"/>
-    <col min="5" max="5" width="15.36328125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="15.08984375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="15.33203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="15.109375" style="1" customWidth="1"/>
     <col min="7" max="7" width="81" style="1" customWidth="1"/>
-    <col min="8" max="8" width="116.36328125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="5.1796875" style="1" customWidth="1"/>
-    <col min="10" max="12" width="14.1796875" style="1" customWidth="1"/>
-    <col min="13" max="13" width="40.36328125" style="1" customWidth="1"/>
-    <col min="14" max="16384" width="8.453125" style="1"/>
+    <col min="8" max="8" width="116.33203125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="5.21875" style="1" customWidth="1"/>
+    <col min="10" max="12" width="14.21875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="40.33203125" style="1" customWidth="1"/>
+    <col min="14" max="16384" width="8.44140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="17.100000000000001" customHeight="1">
@@ -14043,7 +14050,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="156.9" customHeight="1">
+    <row r="2" spans="1:14" ht="156.94999999999999" customHeight="1">
       <c r="A2" s="42" t="s">
         <v>30</v>
       </c>
@@ -14066,7 +14073,7 @@
         <v>50</v>
       </c>
       <c r="H2" s="45" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I2" s="43">
         <v>50</v>
@@ -14333,7 +14340,7 @@
       </c>
       <c r="G11" s="4"/>
       <c r="H11" s="48" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I11" s="25">
         <v>70</v>
@@ -14544,7 +14551,7 @@
       <c r="M18" s="4"/>
       <c r="N18" s="16"/>
     </row>
-    <row r="19" spans="1:14" ht="45.45" customHeight="1">
+    <row r="19" spans="1:14" ht="45.4" customHeight="1">
       <c r="A19" s="9" t="s">
         <v>32</v>
       </c>
@@ -14565,7 +14572,7 @@
       </c>
       <c r="G19" s="4"/>
       <c r="H19" s="49" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I19" s="25">
         <v>90</v>
@@ -14623,11 +14630,11 @@
       <c r="D21" s="9"/>
       <c r="E21" s="53"/>
       <c r="F21" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G21" s="4"/>
       <c r="H21" s="49" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="I21" s="25">
         <v>100</v>
@@ -14717,11 +14724,11 @@
       <c r="D24" s="9"/>
       <c r="E24" s="53"/>
       <c r="F24" s="9" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G24" s="4"/>
       <c r="H24" s="49" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I24" s="25">
         <v>120</v>
@@ -14739,7 +14746,7 @@
         <v>130</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C25" s="9" t="s">
         <v>131</v>
@@ -14775,7 +14782,7 @@
         <v>130</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C26" s="4"/>
       <c r="D26" s="25" t="s">
@@ -14807,11 +14814,11 @@
         <v>130</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C27" s="4"/>
-      <c r="D27" s="25" t="s">
-        <v>135</v>
+      <c r="D27" s="63" t="s">
+        <v>150</v>
       </c>
       <c r="E27" s="53">
         <v>2</v>

</xml_diff>